<commit_message>
Generate precise Buildbooks label PDFs
</commit_message>
<xml_diff>
--- a/apps/buildbooks/database/QAR_Buildbooks_Validation_v0.2.xlsx
+++ b/apps/buildbooks/database/QAR_Buildbooks_Validation_v0.2.xlsx
@@ -1040,7 +1040,7 @@
         <x:v>SHIP</x:v>
       </x:c>
       <x:c r="E4" s="54" t="str">
-        <x:v>Queen Anne's Revenge - Ready-for-Sea Reconstruction, 1718</x:v>
+        <x:v>Queen Anne's Revenge, Frigate, 1718</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -8385,7 +8385,7 @@
         <x:v>QAR-0001</x:v>
       </x:c>
       <x:c r="B4" s="54" t="str">
-        <x:v>Queen Anne's Revenge - Ready-for-Sea Reconstruction, 1718</x:v>
+        <x:v>Queen Anne's Revenge, Frigate, 1718</x:v>
       </x:c>
       <x:c r="C4" s="54" t="str">
         <x:v>QARYARD</x:v>

</xml_diff>